<commit_message>
Incluindo o cadastro dos colaboradores
</commit_message>
<xml_diff>
--- a/Colaboradores.xlsx
+++ b/Colaboradores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Marcacao_Pontos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAEF52C8-9A88-42C5-8B8B-761C991C6A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860E05AA-5B05-4A02-9C09-13BFFB9E78BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Colaborador</t>
   </si>
@@ -46,6 +46,33 @@
   </si>
   <si>
     <t>IORAN RAONE DE ALMEIDA GOIS</t>
+  </si>
+  <si>
+    <t>JOAO ANTONIO PAROCHI</t>
+  </si>
+  <si>
+    <t>JOSE HENRIQUE HERCULANO DE SOUSA</t>
+  </si>
+  <si>
+    <t>KAIC JULIO PEREIRA DE ALMEIDA</t>
+  </si>
+  <si>
+    <t>MARCELINO DONIZETE GUTIERRES</t>
+  </si>
+  <si>
+    <t>09281928817</t>
+  </si>
+  <si>
+    <t>55705342888</t>
+  </si>
+  <si>
+    <t>ROQUE CARLOS NOGUEIRA JUNIOR</t>
+  </si>
+  <si>
+    <t>30895181800</t>
+  </si>
+  <si>
+    <t>MIGUEL AUGUSTO BENEDITO PEREIRA</t>
   </si>
 </sst>
 </file>
@@ -81,16 +108,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -106,8 +146,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{69604D93-BCD2-4854-98C8-8CCF69342EA0}" name="Colaborador" displayName="Colaborador" ref="A1:B6" totalsRowShown="0">
-  <autoFilter ref="A1:B6" xr:uid="{69604D93-BCD2-4854-98C8-8CCF69342EA0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{69604D93-BCD2-4854-98C8-8CCF69342EA0}" name="Colaborador" displayName="Colaborador" ref="A1:B12" totalsRowShown="0">
+  <autoFilter ref="A1:B12" xr:uid="{69604D93-BCD2-4854-98C8-8CCF69342EA0}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{3A376817-B7E2-40A9-91C5-E1E72C0A1033}" name="Colaborador"/>
     <tableColumn id="2" xr3:uid="{C60975E8-7340-4733-B1D0-9BADEAC8F8E1}" name="CPF" dataDxfId="0"/>
@@ -379,10 +419,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -434,10 +474,59 @@
         <v>53677946883</v>
       </c>
     </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1">
+        <v>40513975802</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1">
+        <v>71631436481</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1">
+        <v>39720541814</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>